<commit_message>
implemented features and fix bugs
</commit_message>
<xml_diff>
--- a/Client/public/inventory-update-template.xlsx
+++ b/Client/public/inventory-update-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bikash Prasad\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67EB73-8E25-4E2B-925E-21FA6C392158}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3588B7-40D0-4209-81C2-4E5B8CD8B44E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" xr2:uid="{F7AA387E-76BF-4623-A655-D79100559CC1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10380" xr2:uid="{C8819AD3-DDB1-4A8C-8793-3156AFC06F60}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,100 +25,67 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
-  <si>
-    <t xml:space="preserve">comment </t>
-  </si>
-  <si>
-    <t>employee_code/email</t>
-  </si>
-  <si>
-    <t>inventory_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> asset_tag</t>
-  </si>
-  <si>
-    <t>AST-01034</t>
-  </si>
-  <si>
-    <t>AST-01036</t>
-  </si>
-  <si>
-    <t>AST-01037</t>
-  </si>
-  <si>
-    <t>Assigned</t>
-  </si>
-  <si>
-    <t>In Stock</t>
-  </si>
-  <si>
-    <t>In Repair</t>
-  </si>
-  <si>
-    <t>Retired</t>
-  </si>
-  <si>
-    <t>Lost</t>
-  </si>
-  <si>
-    <t>Disposed</t>
-  </si>
-  <si>
-    <t>AST-01038</t>
-  </si>
-  <si>
-    <t>Asset handover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Updateing the inventory status </t>
-  </si>
-  <si>
-    <t>Send for repai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated,  remove from the list to further use </t>
-  </si>
-  <si>
-    <t>Not in our log, missing</t>
-  </si>
-  <si>
-    <t>AST-01030</t>
-  </si>
-  <si>
-    <t>AST-01028</t>
-  </si>
-  <si>
-    <t>AST-01026</t>
-  </si>
-  <si>
-    <t>EMP0215</t>
-  </si>
-  <si>
-    <t>abhinav.kohli@gmail.com</t>
-  </si>
-  <si>
-    <t>Asset handover to abhi</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+  <si>
+    <t>Employee Id</t>
+  </si>
+  <si>
+    <t>AST-01054</t>
+  </si>
+  <si>
+    <t>inventory status</t>
+  </si>
+  <si>
+    <t>assigned</t>
+  </si>
+  <si>
+    <t>JMV10728</t>
+  </si>
+  <si>
+    <t>Asset Tag</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>assigned to bikash, test bulk inventory status update via sheet</t>
+  </si>
+  <si>
+    <t>in stock</t>
+  </si>
+  <si>
+    <t>AST-01076</t>
+  </si>
+  <si>
+    <t>disposed</t>
+  </si>
+  <si>
+    <t>AST-01074</t>
+  </si>
+  <si>
+    <t>lost</t>
+  </si>
+  <si>
+    <t>AST-01048</t>
+  </si>
+  <si>
+    <t>AST-01070</t>
+  </si>
+  <si>
+    <t>AST-01058</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -148,12 +115,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -468,115 +434,89 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DC2CB05-4AF5-437F-8E40-83D4B2C7F6E9}">
-  <dimension ref="A1:D8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8F10AE-DC2C-4E36-B071-ABCFEBC28653}">
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.21875" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
       <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
+      <c r="C7" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C8" r:id="rId1" xr:uid="{9B216CCA-83DC-42A6-8FB4-AB6C420E41C2}"/>
+    <hyperlink ref="A2" r:id="rId1" display="bikash@jmv.co.in" xr:uid="{10820202-7348-4499-9E34-717F70290301}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix pdf layout break, improve UI, improve Analytics chart for more insights data
</commit_message>
<xml_diff>
--- a/Client/public/inventory-update-template.xlsx
+++ b/Client/public/inventory-update-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bikash Prasad\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3588B7-40D0-4209-81C2-4E5B8CD8B44E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6490F6-982D-4940-A542-DCEE6E6528D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10380" xr2:uid="{C8819AD3-DDB1-4A8C-8793-3156AFC06F60}"/>
   </bookViews>
@@ -25,72 +25,52 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
-  <si>
-    <t>Employee Id</t>
-  </si>
-  <si>
-    <t>AST-01054</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>inventory status</t>
   </si>
   <si>
-    <t>assigned</t>
-  </si>
-  <si>
-    <t>JMV10728</t>
-  </si>
-  <si>
     <t>Asset Tag</t>
   </si>
   <si>
     <t>Comment</t>
   </si>
   <si>
-    <t>assigned to bikash, test bulk inventory status update via sheet</t>
-  </si>
-  <si>
     <t>in stock</t>
   </si>
   <si>
-    <t>AST-01076</t>
-  </si>
-  <si>
     <t>disposed</t>
   </si>
   <si>
-    <t>AST-01074</t>
-  </si>
-  <si>
     <t>lost</t>
   </si>
   <si>
-    <t>AST-01048</t>
-  </si>
-  <si>
-    <t>AST-01070</t>
-  </si>
-  <si>
-    <t>AST-01058</t>
+    <t>JMV-LAP-01054</t>
+  </si>
+  <si>
+    <t>JMV-KBD-01076</t>
+  </si>
+  <si>
+    <t>JMV-LAP-01074</t>
+  </si>
+  <si>
+    <t>JMV-LAP-01048</t>
+  </si>
+  <si>
+    <t>JMV-LAP-01070</t>
+  </si>
+  <si>
+    <t>lost, test bulk inventory status update via sheet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -113,16 +93,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -435,88 +412,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8F10AE-DC2C-4E36-B071-ABCFEBC28653}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.88671875" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="bikash@jmv.co.in" xr:uid="{10820202-7348-4499-9E34-717F70290301}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>